<commit_message>
feat: update figure of guidelines non-complainment
</commit_message>
<xml_diff>
--- a/notebooks/03_e2r_guidelines/table_5_1_guideline_violations.xlsx
+++ b/notebooks/03_e2r_guidelines/table_5_1_guideline_violations.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Avoid parentheses, brackets, and unusual symbols (%, &amp;, /)</t>
+          <t>Parentheses and unusual symbols</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -456,7 +456,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Avoid abstract, technical, or complex terms</t>
+          <t>Abstract or technical terms</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -471,7 +471,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Avoid uppercase letters or words</t>
+          <t>Uppercase letters or words</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -486,7 +486,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Avoid adverbs ending in -mente</t>
+          <t>Adverbs ending in -mente</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -501,7 +501,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Avoid reflexive passive voice</t>
+          <t>Reflexive passive voice</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -516,7 +516,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Avoid passive voice</t>
+          <t>Passive voice</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -531,7 +531,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Avoid abbreviations</t>
+          <t>Abbreviations</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Avoid compound tenses, conditionals, and subjunctives</t>
+          <t>Compound tenses or subjunctives</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -561,7 +561,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Avoid incidental clauses enclosed by commas</t>
+          <t>Incidental clauses (comma-enclosed)</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -576,7 +576,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Avoid acronyms</t>
+          <t>Acronyms</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -591,7 +591,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Simple sentences; avoid complex clauses</t>
+          <t>Overly complex sentence structure</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Use non-sexist language with generic terms</t>
+          <t>Gendered or exclusive language</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -621,7 +621,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Avoid complex connectors (therefore, nevertheless, etc.)</t>
+          <t>Complex connectors</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -636,7 +636,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Do not use "etcetera" or ellipses</t>
+          <t>Etcetera or ellipses</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -651,7 +651,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Avoid gerund constructions</t>
+          <t>Gerund constructions</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -666,7 +666,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Write numbers as digits; explain complex numbers</t>
+          <t>Numbers written as words</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -681,7 +681,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Use simple, frequently-used language</t>
+          <t>Infrequent or complex vocabulary</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -696,7 +696,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Avoid Roman numerals (except centuries, kings, popes)</t>
+          <t>Roman numerals</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -711,7 +711,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Negation must be clear; avoid double negatives</t>
+          <t>Double negatives</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Prefer affirmative sentences</t>
+          <t>Negative sentence phrasing</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -741,7 +741,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Use lists when there are multiple elements</t>
+          <t>Missing list formatting</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -756,7 +756,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Do not present more than two ideas in one sentence</t>
+          <t>Multiple ideas in one sentence</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Do not use quotation marks (unless accompanied by explanation)</t>
+          <t>Unexplained quotation marks</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -786,7 +786,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Separate phone numbers into blocks</t>
+          <t>Unformatted phone numbers</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Avoid words that add no information</t>
+          <t>Redundant or empty words</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -816,7 +816,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Do not use semicolons</t>
+          <t>Semicolons</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -831,7 +831,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Use titles that anticipate content</t>
+          <t>Non-descriptive headings</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Avoid date formats with dashes or slashes</t>
+          <t>Ambiguous date formats</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -861,7 +861,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Address the reader directly when appropriate</t>
+          <t>Indirect reader address</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -876,7 +876,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Avoid fractions and percentages; describe them in words</t>
+          <t>Fractions and percentages</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -891,7 +891,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Avoid foreign-language words if not widely used</t>
+          <t>Uncommon foreign words</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -906,7 +906,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Avoid two or more successive verbs (except periphrases)</t>
+          <t>Successive verb chains</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Avoid impersonal sentences</t>
+          <t>Impersonal sentences</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -936,7 +936,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Use paragraph breaks to separate ideas</t>
+          <t>Missing paragraph breaks</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -951,7 +951,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Avoid vague words (cosa, algo, aspecto)</t>
+          <t>Vague or imprecise words</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Avoid appositions that disrupt reading flow</t>
+          <t>Disruptive appositions</t>
         </is>
       </c>
       <c r="C37" t="n">

</xml_diff>